<commit_message>
Configurando e Centralizando Logs
</commit_message>
<xml_diff>
--- a/input/1.modalidades.xlsx
+++ b/input/1.modalidades.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B9183A-3162-4FCE-80FC-EBECF87DE0A4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>Presencial</t>
   </si>
@@ -50,12 +51,15 @@
   </si>
   <si>
     <t>ENSINO_A_DISTANCIA</t>
+  </si>
+  <si>
+    <t>proparoxitona</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -105,7 +109,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -180,6 +184,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -215,6 +236,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -390,16 +428,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -410,7 +448,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -421,7 +459,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -432,7 +470,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -441,6 +479,17 @@
       </c>
       <c r="C4" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(modalidade): Adicionando a funcionalidade de excluir por planilha
</commit_message>
<xml_diff>
--- a/input/1.modalidades.xlsx
+++ b/input/1.modalidades.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73B9183A-3162-4FCE-80FC-EBECF87DE0A4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{818716D4-7EF6-42DE-8844-9B45135E058E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Presencial</t>
   </si>
@@ -51,9 +51,6 @@
   </si>
   <si>
     <t>ENSINO_A_DISTANCIA</t>
-  </si>
-  <si>
-    <t>proparoxitona</t>
   </si>
 </sst>
 </file>
@@ -429,7 +426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -481,17 +478,6 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
-        <v>2</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>

</xml_diff>